<commit_message>
Modificació de gerbers i power point
</commit_message>
<xml_diff>
--- a/KiCad/Pressupost_PCB_Seients.xlsx
+++ b/KiCad/Pressupost_PCB_Seients.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakar\OneDrive\Documentos\PROJECTE_D_EDD\edd-project-grup-dijous-dj_d_seients\KiCad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B019E9EE-E68F-419A-BCA7-03D5A9CD183D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08BA47CE-452B-4365-B073-BF7384B179DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>